<commit_message>
Populate reference prices from real data, flag when contract-variance is circular
Cannot fabricate real negotiated contract rates in this demo tenant, so instead
of inventing plausible numbers: excel/populate_reference_from_savings.py fills
reference-prices.xlsx with the lowest price already paid per item, pulled from
the already outlier-filtered price-variance groups (10 rows, up from 3 hand-picked
examples).

This makes contract-variance mathematically identical to price-variance when the
reference data is self-derived this way (verified: both totals came back as
exactly $2,765,868.00 on the same run) — added derivedFromInternalData/note
fields to flag this automatically, surfaced in the CLI, dashboard callout, and
Excel export, so the two totals are never presented as independent confirmation
of each other.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014svrhqnnBaWojbrkaBsKx8
</commit_message>
<xml_diff>
--- a/excel/reference-prices.xlsx
+++ b/excel/reference-prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sambit\fusiontest\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{922C965F-A854-4C0C-AFE5-13DB0AE8F7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{90AC640F-F10D-415E-8219-BBAB38535816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{5F68713D-8659-4224-B9D7-A24403B60FE5}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="19200" windowHeight="11170" xr2:uid="{4423A5AB-B279-4029-8537-8101108CFC38}"/>
   </bookViews>
   <sheets>
     <sheet name="Reference Prices" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="31">
   <si>
     <t>Category</t>
   </si>
@@ -71,7 +71,13 @@
     <t>Ea</t>
   </si>
   <si>
-    <t>EXAMPLE — replace with real rate</t>
+    <t>DERIVED — lowest of 4 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
+  </si>
+  <si>
+    <t>Recruiting expenses</t>
+  </si>
+  <si>
+    <t>DERIVED — lowest of 3 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
   </si>
   <si>
     <t>Contractor Expense</t>
@@ -80,10 +86,52 @@
     <t>Outside Contractors</t>
   </si>
   <si>
+    <t>DERIVED — lowest of 24 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
+  </si>
+  <si>
     <t>Marketing General</t>
   </si>
   <si>
     <t>Marketing Expenses</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
+  </si>
+  <si>
+    <t>Therapy - Supplies</t>
+  </si>
+  <si>
+    <t>Cafeteria Subsidies</t>
+  </si>
+  <si>
+    <t>DERIVED — lowest of 5 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
+  </si>
+  <si>
+    <t>962.58 Professional Services</t>
+  </si>
+  <si>
+    <t>Killowatts of Green Energy</t>
+  </si>
+  <si>
+    <t>kWh</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Activities - Entertainment</t>
+  </si>
+  <si>
+    <t>Purchase</t>
+  </si>
+  <si>
+    <t>Housekeeping Supplies</t>
+  </si>
+  <si>
+    <t>Advertising Consulting</t>
+  </si>
+  <si>
+    <t>Hr</t>
   </si>
 </sst>
 </file>
@@ -463,16 +511,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD510E6D-1FE7-4C8B-9670-68210DE07060}">
-  <dimension ref="A1:G4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B456AE3-5398-487C-8B28-841D09A83F6C}">
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="144.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -506,7 +555,7 @@
         <v>7</v>
       </c>
       <c r="D2">
-        <v>1450000</v>
+        <v>1407010</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -523,10 +572,10 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3">
-        <v>15000</v>
+        <v>84680</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -535,7 +584,7 @@
         <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -546,7 +595,7 @@
         <v>14</v>
       </c>
       <c r="D4">
-        <v>12000</v>
+        <v>14204</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
@@ -555,6 +604,146 @@
         <v>9</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5">
+        <v>11321</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6">
+        <v>7744</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>61401</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9">
+        <v>4347</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10">
+        <v>5848</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove all synthetic data from reference-prices.xlsx per explicit no-synthetic-data requirement
reference-prices.xlsx is now headers-only (was: 3 hand-typed example rows,
then later populate_reference_from_savings.py-derived rows). Both were real
enough to be useful for testing the mechanism, but neither is an actual Fusion
system record, and the user explicitly requires demo data come only from the
system. create_reference_template.py no longer contains EXAMPLE_ROWS at all,
so re-running it can't reintroduce fake numbers.

Also made po:analyze accept a window-days CLI arg like the other agents, for
running the 1-year analysis the user requested.

Agreement-price variance (purchaseAgreementLines) is unaffected — it was
already 100% system-sourced and remains the one caveat-free savings signal.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014svrhqnnBaWojbrkaBsKx8
</commit_message>
<xml_diff>
--- a/excel/reference-prices.xlsx
+++ b/excel/reference-prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sambit\fusiontest\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90AC640F-F10D-415E-8219-BBAB38535816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1832260C-2502-473F-94EF-AA5785D52123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="19200" windowHeight="11170" xr2:uid="{4423A5AB-B279-4029-8537-8101108CFC38}"/>
+    <workbookView xWindow="3040" yWindow="3040" windowWidth="19200" windowHeight="11170" xr2:uid="{4423A5AB-B279-4029-8537-8101108CFC38}"/>
   </bookViews>
   <sheets>
     <sheet name="Reference Prices" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Category</t>
   </si>
@@ -60,78 +60,6 @@
   </si>
   <si>
     <t>Notes</t>
-  </si>
-  <si>
-    <t>Business Liability Insurance</t>
-  </si>
-  <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>Ea</t>
-  </si>
-  <si>
-    <t>DERIVED — lowest of 4 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
-  </si>
-  <si>
-    <t>Recruiting expenses</t>
-  </si>
-  <si>
-    <t>DERIVED — lowest of 3 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
-  </si>
-  <si>
-    <t>Contractor Expense</t>
-  </si>
-  <si>
-    <t>Outside Contractors</t>
-  </si>
-  <si>
-    <t>DERIVED — lowest of 24 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
-  </si>
-  <si>
-    <t>Marketing General</t>
-  </si>
-  <si>
-    <t>Marketing Expenses</t>
-  </si>
-  <si>
-    <t>Miscellaneous</t>
-  </si>
-  <si>
-    <t>Therapy - Supplies</t>
-  </si>
-  <si>
-    <t>Cafeteria Subsidies</t>
-  </si>
-  <si>
-    <t>DERIVED — lowest of 5 price(s) paid for this item in the 90-day window as of 2026-08-21. NOT an authoritative negotiated contract rate — replace with a real rate when available.</t>
-  </si>
-  <si>
-    <t>962.58 Professional Services</t>
-  </si>
-  <si>
-    <t>Killowatts of Green Energy</t>
-  </si>
-  <si>
-    <t>kWh</t>
-  </si>
-  <si>
-    <t>Entertainment</t>
-  </si>
-  <si>
-    <t>Activities - Entertainment</t>
-  </si>
-  <si>
-    <t>Purchase</t>
-  </si>
-  <si>
-    <t>Housekeeping Supplies</t>
-  </si>
-  <si>
-    <t>Advertising Consulting</t>
-  </si>
-  <si>
-    <t>Hr</t>
   </si>
 </sst>
 </file>
@@ -512,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B456AE3-5398-487C-8B28-841D09A83F6C}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.1796875" bestFit="1" customWidth="1"/>
@@ -547,206 +475,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>1407010</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>84680</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4">
-        <v>14204</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5">
-        <v>11321</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6">
-        <v>7744</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>61401</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8">
-        <v>15</v>
-      </c>
-      <c r="E8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9">
-        <v>4347</v>
-      </c>
-      <c r="E9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10">
-        <v>5848</v>
-      </c>
-      <c r="E10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11">
-        <v>42</v>
-      </c>
-      <c r="E11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>